<commit_message>
fix: reconcile final deliverables and presentation deck to ground-truth figures
- Synchronize PowerPoint decks (14 slides) to verified deposit liabilities (₹131.09 Cr) and churn balance at risk (₹67.33 Cr / 51.37%)
- Update segment at-risk distribution (Wealth: ₹39.73 Cr, Privileged: ₹19.67 Cr, Mass Retail: ₹7.94 Cr)
- Reconcile frontline archetypes (A-F) and top 5 branch hubs (BR004, BR001, BR023, BR014, BR012)
- Update auditor.py and checklist_builder.py to reflect exact ground truth and regenerate audit workbooks
- Synchronize narrative figures across docs (06, 07, 09, 10, FINAL_README, powerbi/README)
</commit_message>
<xml_diff>
--- a/output/FINAL_SUBMISSION_CHECKLIST.xlsx
+++ b/output/FINAL_SUBMISSION_CHECKLIST.xlsx
@@ -760,7 +760,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>None. 2,402 customers scored High/Very High (₹337.89 Cr exposed).</t>
+          <t>None. 2,402 customers scored High/Very High (₹67.33 Cr exposed).</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -910,17 +910,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Apex_Retail_Bank_Executive_Deck.pptx</t>
+          <t>Apex_Retail_Bank_Executive_Presentation.pptx</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>output/Apex_Retail_Bank_Executive_Deck.pptx &amp; docs/09_executive_story.md</t>
+          <t>output/Apex_Retail_Bank_Executive_Presentation.pptx &amp; docs/09_executive_story.md</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Open in PowerPoint to review slides and presenter notes.</t>
+          <t>Open in PowerPoint to review 14 slides and presenter notes.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>output/Apex_Retail_Bank_Executive_Deck.pptx</t>
+          <t>output/Apex_Retail_Bank_Executive_Presentation.pptx</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open the deck, review the 12 slides and presenter notes before executive delivery.</t>
+          <t>Open the deck, review the 14 slides and presenter notes before executive delivery.</t>
         </is>
       </c>
     </row>

</xml_diff>